<commit_message>
Server implemente new chanesd
</commit_message>
<xml_diff>
--- a/My Projects/Vinayaka Chavithi/server/assets/participants.xlsx
+++ b/My Projects/Vinayaka Chavithi/server/assets/participants.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="34">
   <si>
     <t>Date &amp; Time</t>
   </si>
@@ -107,6 +107,12 @@
   </si>
   <si>
     <t>Games</t>
+  </si>
+  <si>
+    <t>2026-09-05T18:44:26.198Z</t>
+  </si>
+  <si>
+    <t>VInod</t>
   </si>
 </sst>
 </file>
@@ -483,7 +489,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -639,6 +645,32 @@
         <v>31</v>
       </c>
       <c r="H6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7" t="s">
+        <v>18</v>
+      </c>
+      <c r="H7" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>